<commit_message>
cc Email adresses Update
</commit_message>
<xml_diff>
--- a/MoM_Excellence_program2026.xlsx
+++ b/MoM_Excellence_program2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Documents\GitHub\Excellence_Program\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE3C736D-3B65-4E89-96DC-018A2618119E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C7AAB18-59B2-4688-A91A-8F770B44DA0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="71">
   <si>
     <t>Meeting Minutes</t>
   </si>
@@ -201,6 +201,73 @@
   </si>
   <si>
     <t xml:space="preserve"> Hans Ehm, Abdelgafar Ismail, Excellence program Students , Botho Schanze, Tim , Hans ,  Wilfried , Ana</t>
+  </si>
+  <si>
+    <t>24.07.2026</t>
+  </si>
+  <si>
+    <t>Presentation</t>
+  </si>
+  <si>
+    <t>all</t>
+  </si>
+  <si>
+    <t>Feedback info</t>
+  </si>
+  <si>
+    <t>Christelle:
+Crops storage: thank you for the very good updates
+Good that you thought of the most important aspects of the storage
+Did you consider the storage capacity from previous year – and show a status of the capacity in the app</t>
+  </si>
+  <si>
+    <t>Mariata:
+Sales &amp; marketing: thank you for the very good updates
+Good job to research  into what is existing already this is called state of the art – I recommend it as best practice
+Please look at what are the challenges to create an app</t>
+  </si>
+  <si>
+    <t>Tania:
+Face recognition: thank you for the very good updates
+Good job to start with improving and enhancing the previous work – also recommend it as best practive</t>
+  </si>
+  <si>
+    <t>Abdoul:
+Product transform: thank you for the very good updates
+Good job to study and reverse engineer previous solution – data model is very good step as well – please share a screenshot of it next time
+Did you think of how the app should contain the most important aspects of product transformation</t>
+  </si>
+  <si>
+    <t>Ester:
+Plants: thank you for the very good updates
+Good job to review the previous work – do plausi check for the calculation in excel – thank you for fixing the error
+As next step I would recommend to list what are the important aspects of the plants app – you already did first step – think which aspects are needed for which partner downstream in the supply chain</t>
+  </si>
+  <si>
+    <t>Phares:
+Irrigation system: thank you for the very good updates
+Good job to research  into what is existing already this is called state of the art
+I would recommend to focus on designing the app to make more water saving planning</t>
+  </si>
+  <si>
+    <t>Jean-Louis:
+Equipment: thank you for the very good updates
+Good job to research  into what is existing already this is called state of the art
+One of the most important aspects of machine is utilization and maintenance I would recommend to include in the app</t>
+  </si>
+  <si>
+    <t>Aida:
+Not in the call</t>
+  </si>
+  <si>
+    <t>Alix:
+Not in the call</t>
+  </si>
+  <si>
+    <t>Hans and Abdo</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Hans Ehm, Abdelgafar Ismail, Excellence program Students , Botho Schanze, Tim , Hans ,  Wilfried , Ana….</t>
   </si>
 </sst>
 </file>
@@ -370,7 +437,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -430,23 +497,32 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1295,7 +1371,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H20"/>
+  <dimension ref="A1:H30"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="17.453125" style="4" customWidth="1"/>
@@ -1307,16 +1383,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="42.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="21" t="s">
+      <c r="A1" s="24" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="21"/>
-      <c r="C1" s="21"/>
-      <c r="D1" s="21"/>
-      <c r="E1" s="21"/>
-      <c r="F1" s="21"/>
-      <c r="G1" s="21"/>
-      <c r="H1" s="21"/>
+      <c r="B1" s="24"/>
+      <c r="C1" s="24"/>
+      <c r="D1" s="24"/>
+      <c r="E1" s="24"/>
+      <c r="F1" s="24"/>
+      <c r="G1" s="24"/>
+      <c r="H1" s="24"/>
     </row>
     <row r="2" spans="1:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="5"/>
@@ -1425,16 +1501,16 @@
       <c r="H6" s="19"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A7" s="24">
+      <c r="A7" s="21">
         <v>2</v>
       </c>
-      <c r="B7" s="25" t="s">
+      <c r="B7" s="22" t="s">
         <v>30</v>
       </c>
-      <c r="C7" s="25" t="s">
+      <c r="C7" s="22" t="s">
         <v>54</v>
       </c>
-      <c r="D7" s="25" t="s">
+      <c r="D7" s="22" t="s">
         <v>31</v>
       </c>
       <c r="E7" s="20" t="s">
@@ -1443,20 +1519,20 @@
       <c r="F7" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="G7" s="25"/>
-      <c r="H7" s="25"/>
+      <c r="G7" s="22"/>
+      <c r="H7" s="22"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A8" s="24">
+      <c r="A8" s="21">
         <v>3</v>
       </c>
-      <c r="B8" s="25" t="s">
+      <c r="B8" s="22" t="s">
         <v>32</v>
       </c>
-      <c r="C8" s="25" t="s">
+      <c r="C8" s="22" t="s">
         <v>33</v>
       </c>
-      <c r="D8" s="25" t="s">
+      <c r="D8" s="22" t="s">
         <v>34</v>
       </c>
       <c r="E8" s="20" t="s">
@@ -1465,20 +1541,20 @@
       <c r="F8" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="G8" s="25"/>
-      <c r="H8" s="25"/>
+      <c r="G8" s="22"/>
+      <c r="H8" s="22"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A9" s="24">
+      <c r="A9" s="21">
         <v>4</v>
       </c>
-      <c r="B9" s="25" t="s">
+      <c r="B9" s="22" t="s">
         <v>32</v>
       </c>
-      <c r="C9" s="25" t="s">
+      <c r="C9" s="22" t="s">
         <v>36</v>
       </c>
-      <c r="D9" s="25" t="s">
+      <c r="D9" s="22" t="s">
         <v>37</v>
       </c>
       <c r="E9" s="20" t="s">
@@ -1487,20 +1563,20 @@
       <c r="F9" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="G9" s="25"/>
-      <c r="H9" s="25"/>
+      <c r="G9" s="22"/>
+      <c r="H9" s="22"/>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A10" s="24">
+      <c r="A10" s="21">
         <v>5</v>
       </c>
-      <c r="B10" s="25" t="s">
+      <c r="B10" s="22" t="s">
         <v>32</v>
       </c>
-      <c r="C10" s="25" t="s">
+      <c r="C10" s="22" t="s">
         <v>38</v>
       </c>
-      <c r="D10" s="25" t="s">
+      <c r="D10" s="22" t="s">
         <v>39</v>
       </c>
       <c r="E10" s="20" t="s">
@@ -1509,20 +1585,20 @@
       <c r="F10" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="G10" s="25"/>
-      <c r="H10" s="25"/>
+      <c r="G10" s="22"/>
+      <c r="H10" s="22"/>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A11" s="24">
+      <c r="A11" s="21">
         <v>6</v>
       </c>
-      <c r="B11" s="25" t="s">
+      <c r="B11" s="22" t="s">
         <v>32</v>
       </c>
-      <c r="C11" s="25" t="s">
+      <c r="C11" s="22" t="s">
         <v>40</v>
       </c>
-      <c r="D11" s="25" t="s">
+      <c r="D11" s="22" t="s">
         <v>41</v>
       </c>
       <c r="E11" s="20" t="s">
@@ -1531,20 +1607,20 @@
       <c r="F11" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="G11" s="25"/>
-      <c r="H11" s="25"/>
+      <c r="G11" s="22"/>
+      <c r="H11" s="22"/>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A12" s="24">
+      <c r="A12" s="21">
         <v>7</v>
       </c>
-      <c r="B12" s="25" t="s">
+      <c r="B12" s="22" t="s">
         <v>32</v>
       </c>
-      <c r="C12" s="25" t="s">
+      <c r="C12" s="22" t="s">
         <v>42</v>
       </c>
-      <c r="D12" s="25" t="s">
+      <c r="D12" s="22" t="s">
         <v>43</v>
       </c>
       <c r="E12" s="20" t="s">
@@ -1553,20 +1629,20 @@
       <c r="F12" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="G12" s="25"/>
-      <c r="H12" s="25"/>
+      <c r="G12" s="22"/>
+      <c r="H12" s="22"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A13" s="24">
+      <c r="A13" s="21">
         <v>8</v>
       </c>
-      <c r="B13" s="25" t="s">
+      <c r="B13" s="22" t="s">
         <v>32</v>
       </c>
-      <c r="C13" s="25" t="s">
+      <c r="C13" s="22" t="s">
         <v>44</v>
       </c>
-      <c r="D13" s="25" t="s">
+      <c r="D13" s="22" t="s">
         <v>45</v>
       </c>
       <c r="E13" s="20" t="s">
@@ -1575,20 +1651,20 @@
       <c r="F13" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="G13" s="25"/>
-      <c r="H13" s="25"/>
+      <c r="G13" s="22"/>
+      <c r="H13" s="22"/>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A14" s="24">
+      <c r="A14" s="21">
         <v>9</v>
       </c>
-      <c r="B14" s="25" t="s">
+      <c r="B14" s="22" t="s">
         <v>32</v>
       </c>
-      <c r="C14" s="25" t="s">
+      <c r="C14" s="22" t="s">
         <v>46</v>
       </c>
-      <c r="D14" s="25" t="s">
+      <c r="D14" s="22" t="s">
         <v>47</v>
       </c>
       <c r="E14" s="20" t="s">
@@ -1597,20 +1673,20 @@
       <c r="F14" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="G14" s="25"/>
-      <c r="H14" s="25"/>
+      <c r="G14" s="22"/>
+      <c r="H14" s="22"/>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A15" s="24">
+      <c r="A15" s="21">
         <v>10</v>
       </c>
-      <c r="B15" s="25" t="s">
+      <c r="B15" s="22" t="s">
         <v>32</v>
       </c>
-      <c r="C15" s="25" t="s">
+      <c r="C15" s="22" t="s">
         <v>48</v>
       </c>
-      <c r="D15" s="25" t="s">
+      <c r="D15" s="22" t="s">
         <v>49</v>
       </c>
       <c r="E15" s="20" t="s">
@@ -1619,20 +1695,20 @@
       <c r="F15" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="G15" s="25"/>
-      <c r="H15" s="25"/>
+      <c r="G15" s="22"/>
+      <c r="H15" s="22"/>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A16" s="24">
+      <c r="A16" s="21">
         <v>11</v>
       </c>
-      <c r="B16" s="25" t="s">
+      <c r="B16" s="22" t="s">
         <v>32</v>
       </c>
-      <c r="C16" s="25" t="s">
+      <c r="C16" s="22" t="s">
         <v>50</v>
       </c>
-      <c r="D16" s="25" t="s">
+      <c r="D16" s="22" t="s">
         <v>51</v>
       </c>
       <c r="E16" s="20" t="s">
@@ -1641,37 +1717,304 @@
       <c r="F16" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="G16" s="25"/>
-      <c r="H16" s="25"/>
+      <c r="G16" s="22"/>
+      <c r="H16" s="22"/>
     </row>
     <row r="17" spans="1:8" ht="87" x14ac:dyDescent="0.35">
-      <c r="A17" s="24">
+      <c r="A17" s="21">
         <v>12</v>
       </c>
-      <c r="B17" s="26" t="s">
+      <c r="B17" s="23" t="s">
         <v>35</v>
       </c>
-      <c r="C17" s="25" t="s">
+      <c r="C17" s="22" t="s">
         <v>52</v>
       </c>
-      <c r="D17" s="26" t="s">
+      <c r="D17" s="23" t="s">
         <v>53</v>
       </c>
-      <c r="E17" s="25"/>
+      <c r="E17" s="22"/>
       <c r="F17" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="G17" s="25"/>
-      <c r="H17" s="25"/>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A18" s="23"/>
+      <c r="G17" s="22"/>
+      <c r="H17" s="22"/>
+    </row>
+    <row r="18" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+      <c r="A18" s="8">
+        <v>2</v>
+      </c>
+      <c r="B18" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="C18" s="15" t="s">
+        <v>70</v>
+      </c>
+      <c r="D18" s="17" t="s">
+        <v>10</v>
+      </c>
+      <c r="E18" s="16" t="s">
+        <v>11</v>
+      </c>
+      <c r="F18" s="12"/>
+      <c r="G18" s="13"/>
+      <c r="H18" s="14"/>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A19" s="23"/>
+      <c r="A19" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="B19" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="C19" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="D19" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="E19" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="F19" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="G19" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="H19" s="10" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A20" s="23"/>
+      <c r="A20" s="1">
+        <v>1</v>
+      </c>
+      <c r="B20" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="C20" s="18" t="s">
+        <v>57</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="E20" s="20" t="s">
+        <v>17</v>
+      </c>
+      <c r="F20" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="G20" s="18"/>
+      <c r="H20" s="19"/>
+    </row>
+    <row r="21" spans="1:8" ht="87" x14ac:dyDescent="0.35">
+      <c r="A21" s="21">
+        <v>2</v>
+      </c>
+      <c r="B21" s="22" t="s">
+        <v>59</v>
+      </c>
+      <c r="C21" s="22" t="s">
+        <v>60</v>
+      </c>
+      <c r="D21" s="22" t="s">
+        <v>69</v>
+      </c>
+      <c r="E21" s="20" t="s">
+        <v>17</v>
+      </c>
+      <c r="F21" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="G21" s="22"/>
+      <c r="H21" s="22"/>
+    </row>
+    <row r="22" spans="1:8" ht="87" x14ac:dyDescent="0.35">
+      <c r="A22" s="21">
+        <v>3</v>
+      </c>
+      <c r="B22" s="22" t="s">
+        <v>59</v>
+      </c>
+      <c r="C22" s="22" t="s">
+        <v>61</v>
+      </c>
+      <c r="D22" s="22" t="s">
+        <v>69</v>
+      </c>
+      <c r="E22" s="20" t="s">
+        <v>17</v>
+      </c>
+      <c r="F22" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="G22" s="22"/>
+      <c r="H22" s="22"/>
+    </row>
+    <row r="23" spans="1:8" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="A23" s="21">
+        <v>4</v>
+      </c>
+      <c r="B23" s="22" t="s">
+        <v>59</v>
+      </c>
+      <c r="C23" s="22" t="s">
+        <v>62</v>
+      </c>
+      <c r="D23" s="22" t="s">
+        <v>69</v>
+      </c>
+      <c r="E23" s="20" t="s">
+        <v>17</v>
+      </c>
+      <c r="F23" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="G23" s="22"/>
+      <c r="H23" s="22"/>
+    </row>
+    <row r="24" spans="1:8" ht="101.5" x14ac:dyDescent="0.35">
+      <c r="A24" s="21">
+        <v>5</v>
+      </c>
+      <c r="B24" s="22" t="s">
+        <v>59</v>
+      </c>
+      <c r="C24" s="22" t="s">
+        <v>63</v>
+      </c>
+      <c r="D24" s="22" t="s">
+        <v>69</v>
+      </c>
+      <c r="E24" s="20" t="s">
+        <v>17</v>
+      </c>
+      <c r="F24" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="G24" s="22"/>
+      <c r="H24" s="22"/>
+    </row>
+    <row r="25" spans="1:8" ht="116" x14ac:dyDescent="0.35">
+      <c r="A25" s="21">
+        <v>6</v>
+      </c>
+      <c r="B25" s="22" t="s">
+        <v>59</v>
+      </c>
+      <c r="C25" s="22" t="s">
+        <v>64</v>
+      </c>
+      <c r="D25" s="22" t="s">
+        <v>69</v>
+      </c>
+      <c r="E25" s="20" t="s">
+        <v>17</v>
+      </c>
+      <c r="F25" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="G25" s="22"/>
+      <c r="H25" s="22"/>
+    </row>
+    <row r="26" spans="1:8" ht="101.5" x14ac:dyDescent="0.35">
+      <c r="A26" s="21">
+        <v>7</v>
+      </c>
+      <c r="B26" s="22" t="s">
+        <v>59</v>
+      </c>
+      <c r="C26" s="22" t="s">
+        <v>65</v>
+      </c>
+      <c r="D26" s="22" t="s">
+        <v>69</v>
+      </c>
+      <c r="E26" s="20" t="s">
+        <v>17</v>
+      </c>
+      <c r="F26" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="G26" s="22"/>
+      <c r="H26" s="22"/>
+    </row>
+    <row r="27" spans="1:8" ht="101.5" x14ac:dyDescent="0.35">
+      <c r="A27" s="21">
+        <v>8</v>
+      </c>
+      <c r="B27" s="22" t="s">
+        <v>59</v>
+      </c>
+      <c r="C27" s="22" t="s">
+        <v>66</v>
+      </c>
+      <c r="D27" s="22" t="s">
+        <v>69</v>
+      </c>
+      <c r="E27" s="20" t="s">
+        <v>17</v>
+      </c>
+      <c r="F27" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="G27" s="22"/>
+      <c r="H27" s="22"/>
+    </row>
+    <row r="28" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A28" s="21">
+        <v>9</v>
+      </c>
+      <c r="B28" s="22" t="s">
+        <v>59</v>
+      </c>
+      <c r="C28" s="22" t="s">
+        <v>67</v>
+      </c>
+      <c r="D28" s="22" t="s">
+        <v>69</v>
+      </c>
+      <c r="E28" s="20" t="s">
+        <v>17</v>
+      </c>
+      <c r="F28" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="G28" s="22"/>
+      <c r="H28" s="22"/>
+    </row>
+    <row r="29" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A29" s="21">
+        <v>10</v>
+      </c>
+      <c r="B29" s="22" t="s">
+        <v>59</v>
+      </c>
+      <c r="C29" s="22" t="s">
+        <v>68</v>
+      </c>
+      <c r="D29" s="22" t="s">
+        <v>69</v>
+      </c>
+      <c r="E29" s="20" t="s">
+        <v>17</v>
+      </c>
+      <c r="F29" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="G29" s="22"/>
+      <c r="H29" s="22"/>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A30" s="26"/>
+      <c r="B30" s="27"/>
+      <c r="C30" s="27"/>
+      <c r="D30" s="27"/>
+      <c r="E30" s="28"/>
+      <c r="F30" s="29"/>
+      <c r="G30" s="27"/>
+      <c r="H30" s="27"/>
     </row>
   </sheetData>
   <autoFilter ref="A3:H6" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
@@ -1691,7 +2034,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F6:F17" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F6:F17 F20:F30" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>Status</formula1>
     </dataValidation>
   </dataValidations>
@@ -1711,16 +2054,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="37.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="22" t="s">
+      <c r="A1" s="25" t="s">
         <v>20</v>
       </c>
-      <c r="B1" s="22"/>
-      <c r="C1" s="22"/>
-      <c r="D1" s="22"/>
-      <c r="E1" s="22"/>
-      <c r="F1" s="22"/>
-      <c r="G1" s="22"/>
-      <c r="H1" s="22"/>
+      <c r="B1" s="25"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
+      <c r="E1" s="25"/>
+      <c r="F1" s="25"/>
+      <c r="G1" s="25"/>
+      <c r="H1" s="25"/>
     </row>
     <row r="2" spans="1:8" ht="51.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
@@ -1878,18 +2221,18 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1909,18 +2252,18 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{796D9FC9-4B98-4FFD-BB78-C2E8DE274F9F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{099BC07E-159D-4A16-BA20-897EF5E09C4C}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{796D9FC9-4B98-4FFD-BB78-C2E8DE274F9F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>